<commit_message>
Atualiza BACKLOG.xlsx — Issue # da Onda 1 preenchidos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -753,7 +753,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#13</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#14</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#15</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#16</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#17</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#18</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#19</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#20</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#21</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#22</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#23</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>#24</t>
         </is>
       </c>
     </row>

</xml_diff>